<commit_message>
Rename documentation files for clarity and update chord reference
</commit_message>
<xml_diff>
--- a/help/sh-chords.xlsx
+++ b/help/sh-chords.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ed/Projects/Lilypond/help/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B857021F-17D6-1540-867C-59146B38AF52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8625A85-0371-B246-AF43-A8A6BF01E332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="17380" xr2:uid="{35497F95-371D-054C-8979-971CA2FD12C1}"/>
   </bookViews>
@@ -2382,7 +2382,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2412,7 +2412,7 @@
     <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2439,34 +2439,37 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
@@ -3002,141 +3005,141 @@
       <c r="A12" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="C12" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="D12" s="20" t="s">
+      <c r="D12" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="E12" s="20" t="s">
+      <c r="E12" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="F12" s="20" t="s">
+      <c r="F12" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="G12" s="20" t="s">
+      <c r="G12" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="H12" s="20" t="s">
+      <c r="H12" s="22" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A13" s="21"/>
-      <c r="B13" s="22" t="s">
+      <c r="A13" s="23"/>
+      <c r="B13" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="23" t="s">
+      <c r="D13" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="E13" s="23" t="s">
+      <c r="E13" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="F13" s="23" t="s">
+      <c r="F13" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="G13" s="23" t="s">
+      <c r="G13" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="H13" s="24" t="s">
+      <c r="H13" s="25" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A14" s="25"/>
-      <c r="B14" s="26" t="s">
+      <c r="A14" s="15"/>
+      <c r="B14" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="27"/>
-      <c r="D14" s="27"/>
-      <c r="E14" s="23" t="s">
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="F14" s="28" t="s">
+      <c r="F14" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="G14" s="27"/>
-      <c r="H14" s="27"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="26"/>
     </row>
     <row r="15" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A15" s="25"/>
-      <c r="B15" s="27"/>
-      <c r="C15" s="23" t="s">
+      <c r="A15" s="15"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="D15" s="26" t="s">
+      <c r="D15" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="E15" s="27"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="22" t="s">
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="H15" s="23" t="s">
+      <c r="H15" s="27" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A16" s="25"/>
-      <c r="B16" s="23" t="s">
+      <c r="A16" s="15"/>
+      <c r="B16" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="25"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="26" t="s">
+      <c r="C16" s="17"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="F16" s="26" t="s">
+      <c r="F16" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="G16" s="23" t="s">
+      <c r="G16" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="H16" s="26" t="s">
+      <c r="H16" s="29" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A17" s="25"/>
-      <c r="B17" s="26" t="s">
+      <c r="A17" s="15"/>
+      <c r="B17" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="19"/>
     </row>
     <row r="18" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A18" s="25"/>
-      <c r="B18" s="23" t="s">
+      <c r="A18" s="15"/>
+      <c r="B18" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="29"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="25"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="19"/>
     </row>
     <row r="19" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A19" s="25"/>
-      <c r="B19" s="23" t="s">
+      <c r="A19" s="15"/>
+      <c r="B19" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="C19" s="25"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="25"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="19"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>

</xml_diff>